<commit_message>
fix: correção de bug
</commit_message>
<xml_diff>
--- a/dataset.xlsx
+++ b/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sesibahia-my.sharepoint.com/personal/anderson_pereira_fieb_org_br/Documents/Inteligência de Mercado/Data Science/DeploymentML/dsim-recomendacao-de-curso/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_5375D2B3D3305619A922D6F0505ED87656CF24F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D801C6C-00B3-4A59-960B-D8EE9780B031}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="11_5375D2B3D3305619A922D6F0505ED87656CF24F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CC6C6D9-D959-4A4F-816C-C992F6787D4E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="63">
   <si>
     <t>ANO</t>
   </si>
@@ -202,13 +202,33 @@
   <si>
     <t>JACOBINA</t>
   </si>
+  <si>
+    <t>CONCORRÊNCIA (INEP)</t>
+  </si>
+  <si>
+    <t>EMPRESAS (RAIS)</t>
+  </si>
+  <si>
+    <t>SALÁRIO MÉDIO (CAGED)</t>
+  </si>
+  <si>
+    <t>SALDO EMPREGO (CAGED)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -236,9 +256,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10671,36 +10692,36 @@
     <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.08984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>